<commit_message>
update to pces v0.0.17
</commit_message>
<xml_diff>
--- a/embedded/xlsx/embedded-model-exp.xlsx
+++ b/embedded/xlsx/embedded-model-exp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicol/Dropbox/github-repos/pcesbld/xlsxPCES/examples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicol/Dropbox/github-repos/pcesapps/embedded/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59077688-0C7F-C543-AE49-CC75CE0BCF3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C367A948-CD59-5D4E-880B-1626C7C9FEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16840" yWindow="780" windowWidth="24640" windowHeight="18040" activeTab="4" xr2:uid="{7E753834-245C-A346-8630-DEF93455D7FF}"/>
+    <workbookView xWindow="36680" yWindow="3620" windowWidth="31480" windowHeight="20520" activeTab="1" xr2:uid="{7E753834-245C-A346-8630-DEF93455D7FF}"/>
   </bookViews>
   <sheets>
     <sheet name="topo" sheetId="1" r:id="rId1"/>

</xml_diff>